<commit_message>
Revised blood flows to have mass balance while matching liver and kidney flow rates used by Loccisano.
</commit_message>
<xml_diff>
--- a/Inputs/PFOS_template_parameters_Model.xlsx
+++ b/Inputs/PFOS_template_parameters_Model.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/bernstein_amanda_epa_gov/Documents/Documents/PKWG_models/pbpk_template_project/Inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/schlosser_paul_epa_gov/Documents/mcsim-5.6.5/PBPK_Model_Template_Mod/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="39" documentId="13_ncr:1_{B8500040-1252-468E-B7FB-E947D0A7FECC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A51B12B0-07D8-465F-AC83-2FF518B6853C}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="13_ncr:1_{B8500040-1252-468E-B7FB-E947D0A7FECC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88A12944-9953-47C8-9A0F-6B3B2D26F029}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
+    <workbookView xWindow="1830" yWindow="1890" windowWidth="21600" windowHeight="12585" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
   </bookViews>
   <sheets>
     <sheet name="M3MOralBW" sheetId="9" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="239">
   <si>
     <t>Code</t>
   </si>
@@ -741,6 +741,15 @@
   </si>
   <si>
     <t>num.blood.comp</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>plasma</t>
+  </si>
+  <si>
+    <t>Fractions of total plasma flow</t>
   </si>
 </sst>
 </file>
@@ -756,7 +765,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -766,6 +775,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -782,11 +797,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -866,9 +882,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -906,7 +922,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1012,7 +1028,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1154,7 +1170,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1162,19 +1178,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ADCAA70-43B6-4F02-AE2A-67A6EACE5958}">
-  <dimension ref="A1:F104"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:G104"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="51" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.08984375" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.54296875" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" customWidth="1"/>
+    <col min="5" max="5" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1194,7 +1210,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -1208,7 +1224,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1219,7 +1235,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1230,7 +1246,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -1247,7 +1263,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -1264,7 +1280,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -1278,7 +1294,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>20</v>
       </c>
@@ -1292,7 +1308,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>235</v>
       </c>
@@ -1309,7 +1325,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>136</v>
       </c>
@@ -1326,7 +1342,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>137</v>
       </c>
@@ -1343,7 +1359,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>180</v>
       </c>
@@ -1360,7 +1376,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>184</v>
       </c>
@@ -1377,7 +1393,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>169</v>
       </c>
@@ -1394,7 +1410,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>198</v>
       </c>
@@ -1406,13 +1422,13 @@
       </c>
       <c r="E15">
         <f>1-SUM(E76:E85)</f>
-        <v>7.0500000000000118E-2</v>
+        <v>0</v>
       </c>
       <c r="F15" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>201</v>
       </c>
@@ -1427,7 +1443,7 @@
         <v>0.84000000000000008</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>0</v>
       </c>
@@ -1444,7 +1460,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>71</v>
       </c>
@@ -1461,7 +1477,7 @@
         <v>500.13</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>27</v>
       </c>
@@ -1475,7 +1491,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>29</v>
       </c>
@@ -1489,7 +1505,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>227</v>
       </c>
@@ -1507,7 +1523,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>31</v>
       </c>
@@ -1521,7 +1537,7 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>33</v>
       </c>
@@ -1534,26 +1550,36 @@
       <c r="D24">
         <v>0</v>
       </c>
-      <c r="E24">
+      <c r="E24" s="4">
+        <f>F25*(1-E52)</f>
+        <v>7.0270200000000003</v>
+      </c>
+      <c r="F24" s="4">
+        <v>14</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" t="s">
+        <v>44</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="F25" s="4">
         <f>F24*(1-E99)</f>
         <v>7.5600000000000005</v>
       </c>
-      <c r="F24">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B25" t="s">
-        <v>44</v>
-      </c>
-      <c r="D25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G25" s="4" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>142</v>
       </c>
@@ -1570,7 +1596,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>143</v>
       </c>
@@ -1587,7 +1613,7 @@
         <v>16.7</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>48</v>
       </c>
@@ -1604,7 +1630,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>144</v>
       </c>
@@ -1621,7 +1647,7 @@
         <v>2E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>145</v>
       </c>
@@ -1635,7 +1661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>146</v>
       </c>
@@ -1652,7 +1678,7 @@
         <v>8.0000000000000002E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>52</v>
       </c>
@@ -1666,7 +1692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>53</v>
       </c>
@@ -1683,7 +1709,7 @@
         <v>25.1</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>54</v>
       </c>
@@ -1697,7 +1723,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>55</v>
       </c>
@@ -1714,7 +1740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>170</v>
       </c>
@@ -1728,7 +1754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>57</v>
       </c>
@@ -1745,7 +1771,7 @@
         <v>634.5</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>224</v>
       </c>
@@ -1762,7 +1788,7 @@
         <v>3.5999999999999999E-3</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>225</v>
       </c>
@@ -1779,7 +1805,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>226</v>
       </c>
@@ -1796,7 +1822,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>147</v>
       </c>
@@ -1810,7 +1836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>148</v>
       </c>
@@ -1824,7 +1850,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>149</v>
       </c>
@@ -1838,7 +1864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>150</v>
       </c>
@@ -1852,7 +1878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>151</v>
       </c>
@@ -1866,7 +1892,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>152</v>
       </c>
@@ -1880,7 +1906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>153</v>
       </c>
@@ -1894,7 +1920,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>154</v>
       </c>
@@ -1908,7 +1934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>38</v>
       </c>
@@ -1919,7 +1945,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>173</v>
       </c>
@@ -1930,7 +1956,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>40</v>
       </c>
@@ -1941,7 +1967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>190</v>
       </c>
@@ -1958,7 +1984,7 @@
         <v>7.0499999999999993E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>165</v>
       </c>
@@ -1972,7 +1998,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>166</v>
       </c>
@@ -1983,7 +2009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>204</v>
       </c>
@@ -1997,7 +2023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>206</v>
       </c>
@@ -2011,7 +2037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>230</v>
       </c>
@@ -2028,7 +2054,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>42</v>
       </c>
@@ -2042,7 +2068,7 @@
         <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>0</v>
       </c>
@@ -2059,7 +2085,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>81</v>
       </c>
@@ -2076,7 +2102,7 @@
         <v>3.1199999999999999E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>138</v>
       </c>
@@ -2090,7 +2116,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>140</v>
       </c>
@@ -2104,7 +2130,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>84</v>
       </c>
@@ -2118,7 +2144,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>91</v>
       </c>
@@ -2132,7 +2158,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>92</v>
       </c>
@@ -2149,7 +2175,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>93</v>
       </c>
@@ -2166,7 +2192,7 @@
         <v>8.3999999999999995E-3</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>94</v>
       </c>
@@ -2183,7 +2209,7 @@
         <v>8.4000000000000003E-4</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>95</v>
       </c>
@@ -2197,7 +2223,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>96</v>
       </c>
@@ -2211,7 +2237,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>97</v>
       </c>
@@ -2225,7 +2251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>98</v>
       </c>
@@ -2239,7 +2265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>99</v>
       </c>
@@ -2253,7 +2279,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>100</v>
       </c>
@@ -2267,7 +2293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>155</v>
       </c>
@@ -2285,7 +2311,7 @@
         <v>0.76456000000000002</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>106</v>
       </c>
@@ -2299,7 +2325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>107</v>
       </c>
@@ -2312,11 +2338,18 @@
       <c r="D77">
         <v>0</v>
       </c>
-      <c r="E77">
+      <c r="E77" s="4">
+        <f>F77/(1-E$52)</f>
+        <v>0.19688004303388917</v>
+      </c>
+      <c r="F77" s="4">
         <v>0.183</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G77" s="4" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>108</v>
       </c>
@@ -2329,11 +2362,19 @@
       <c r="D78">
         <v>0</v>
       </c>
-      <c r="E78">
+      <c r="E78" s="4">
+        <f>F78/(1-E$52)</f>
+        <v>0.15169445938676707</v>
+      </c>
+      <c r="F78" s="4">
         <v>0.14099999999999999</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G78" s="4">
+        <f>F78*F25-E78*E24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>109</v>
       </c>
@@ -2347,7 +2388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>110</v>
       </c>
@@ -2361,7 +2402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>111</v>
       </c>
@@ -2375,7 +2416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>112</v>
       </c>
@@ -2389,7 +2430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>113</v>
       </c>
@@ -2403,7 +2444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>114</v>
       </c>
@@ -2417,7 +2458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>158</v>
       </c>
@@ -2430,12 +2471,12 @@
       <c r="D85">
         <v>0</v>
       </c>
-      <c r="E85">
-        <f>1-E77-E78-E52</f>
-        <v>0.60549999999999993</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E85" s="4">
+        <f>1-E77-E78</f>
+        <v>0.65142549757934376</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>123</v>
       </c>
@@ -2446,7 +2487,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>124</v>
       </c>
@@ -2457,7 +2498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>125</v>
       </c>
@@ -2471,7 +2512,7 @@
         <v>3.72</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>126</v>
       </c>
@@ -2485,7 +2526,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>127</v>
       </c>
@@ -2496,7 +2537,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>128</v>
       </c>
@@ -2507,7 +2548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>129</v>
       </c>
@@ -2518,7 +2559,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>130</v>
       </c>
@@ -2529,7 +2570,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>131</v>
       </c>
@@ -2540,7 +2581,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>132</v>
       </c>
@@ -2551,7 +2592,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>161</v>
       </c>
@@ -2565,7 +2606,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>0</v>
       </c>
@@ -2582,7 +2623,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>35</v>
       </c>
@@ -2593,7 +2634,7 @@
         <v>0.46</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>0</v>
       </c>
@@ -2608,7 +2649,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>75</v>
       </c>
@@ -2616,7 +2657,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>77</v>
       </c>
@@ -2624,7 +2665,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>79</v>
       </c>
@@ -2662,6 +2703,51 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
+    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </j747ac98061d40f0aa7bd47e1db5675d>
+    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
+    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
+    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
+    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creator>
+    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </EPA_x0020_Contributor>
+    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </e3f09c3df709400db2417a7161762d62>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5efa0b4590ceb4068c523eef838cbf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d32b47d5805bf9e4ccfb00021215c68" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3134,52 +3220,12 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
-    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </j747ac98061d40f0aa7bd47e1db5675d>
-    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
-    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
-    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
-    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creator>
-    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </EPA_x0020_Contributor>
-    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </e3f09c3df709400db2417a7161762d62>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -3188,16 +3234,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0DBE9A74-1F37-44E9-8DD1-1B9BE601B589}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3207,22 +3244,46 @@
     <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
     <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0DBE9A74-1F37-44E9-8DD1-1B9BE601B589}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
+    <ds:schemaRef ds:uri="41d9f072-86bf-4c63-b117-debf50ff4701"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>